<commit_message>
feat: refine web demo, add test suite and weekly report generation
- Improved hybrid decision strategy for higher classification accuracy
- Dark mode and layout polish for the three-pane support UI
- pytest coverage for cleaning / classification / extraction
- Weekly operations report export pipeline
</commit_message>
<xml_diff>
--- a/data/mock_100_已分析.xlsx
+++ b/data/mock_100_已分析.xlsx
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.67</v>
+        <v>0.703</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -560,7 +560,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.67</v>
+        <v>0.679</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -984,7 +984,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1163,15 +1163,15 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>客服态度差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.67</v>
+        <v>0.623</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>已读不回</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1181,22 +1181,22 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>您好，感谢您的反馈。关于“已读不回”问题，我们已记录并将对客服进行培训并由主管1小时内回访您，给您带来不便深表歉意，感谢您的监督。</t>
+          <t>您好，感谢您的反馈。关于“货不对版”问题，我们已记录并将核对仓储记录并补发正确商品，给您带来不便深表歉意，感谢您的监督。</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>非常理解您的心情，已读不回确实让人失望。我们已加急处理，会对客服进行培训并由主管1小时内回访您，希望能再给我们一次弥补的机会～</t>
+          <t>非常理解您的心情，货不对版确实让人失望。我们已加急处理，会核对仓储记录并补发正确商品，希望能再给我们一次弥补的机会～</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>哎呀让您踩坑了！已读不回这锅我们背，已安排对客服进行培训并由主管1小时内回访您，小客服在线等您验收，祝您接下来体验加分～</t>
+          <t>哎呀让您踩坑了！货不对版这锅我们背，已安排核对仓储记录并补发正确商品，小客服在线等您验收，祝您接下来体验加分～</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>bge</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.67</v>
+        <v>0.703</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.67</v>
+        <v>0.696</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1375,15 +1375,15 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>质量差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.35</v>
+        <v>0.7</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>质量差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1393,22 +1393,22 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>您好，感谢您的反馈。关于“质量差”问题，我们已记录并将安排质检复核并支持免费换新/退货，给您带来不便深表歉意，感谢您的监督。</t>
+          <t>您好，感谢您的反馈。关于“货不对版”问题，我们已记录并将核对仓储记录并补发正确商品，给您带来不便深表歉意，感谢您的监督。</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>非常理解您的心情，质量差确实让人失望。我们已加急处理，会安排质检复核并支持免费换新/退货，希望能再给我们一次弥补的机会～</t>
+          <t>非常理解您的心情，货不对版确实让人失望。我们已加急处理，会核对仓储记录并补发正确商品，希望能再给我们一次弥补的机会～</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>哎呀让您踩坑了！质量差这锅我们背，已安排安排质检复核并支持免费换新/退货，小客服在线等您验收，祝您接下来体验加分～</t>
+          <t>哎呀让您踩坑了！货不对版这锅我们背，已安排核对仓储记录并补发正确商品，小客服在线等您验收，祝您接下来体验加分～</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>bge</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.67</v>
+        <v>0.741</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.67</v>
+        <v>0.696</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2064,15 +2064,15 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>质量差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.35</v>
+        <v>0.665</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>质量差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2082,22 +2082,22 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>您好，感谢您的反馈。关于“质量差”问题，我们已记录并将安排质检复核并支持免费换新/退货，给您带来不便深表歉意，感谢您的监督。</t>
+          <t>您好，感谢您的反馈。关于“货不对版”问题，我们已记录并将核对仓储记录并补发正确商品，给您带来不便深表歉意，感谢您的监督。</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>非常理解您的心情，质量差确实让人失望。我们已加急处理，会安排质检复核并支持免费换新/退货，希望能再给我们一次弥补的机会～</t>
+          <t>非常理解您的心情，货不对版确实让人失望。我们已加急处理，会核对仓储记录并补发正确商品，希望能再给我们一次弥补的机会～</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>哎呀让您踩坑了！质量差这锅我们背，已安排安排质检复核并支持免费换新/退货，小客服在线等您验收，祝您接下来体验加分～</t>
+          <t>哎呀让您踩坑了！货不对版这锅我们背，已安排核对仓储记录并补发正确商品，小客服在线等您验收，祝您接下来体验加分～</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>bge</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.67</v>
+        <v>0.678</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.67</v>
+        <v>0.716</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2704,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.67</v>
+        <v>0.671</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2916,7 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.67</v>
+        <v>0.696</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3022,7 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0.67</v>
+        <v>0.722</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3124,15 +3124,15 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>客服态度差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0.67</v>
+        <v>0.65</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>已读不回</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -3142,22 +3142,22 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>您好，感谢您的反馈。关于“已读不回”问题，我们已记录并将对客服进行培训并由主管1小时内回访您，给您带来不便深表歉意，感谢您的监督。</t>
+          <t>您好，感谢您的反馈。关于“货不对版”问题，我们已记录并将核对仓储记录并补发正确商品，给您带来不便深表歉意，感谢您的监督。</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>非常理解您的心情，已读不回确实让人失望。我们已加急处理，会对客服进行培训并由主管1小时内回访您，希望能再给我们一次弥补的机会～</t>
+          <t>非常理解您的心情，货不对版确实让人失望。我们已加急处理，会核对仓储记录并补发正确商品，希望能再给我们一次弥补的机会～</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>哎呀让您踩坑了！已读不回这锅我们背，已安排对客服进行培训并由主管1小时内回访您，小客服在线等您验收，祝您接下来体验加分～</t>
+          <t>哎呀让您踩坑了！货不对版这锅我们背，已安排核对仓储记录并补发正确商品，小客服在线等您验收，祝您接下来体验加分～</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>bge</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3230,15 +3230,15 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>质量差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.67</v>
+        <v>0.636</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>质量差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -3248,22 +3248,22 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>您好，感谢您的反馈。关于“质量差”问题，我们已记录并将安排质检复核并支持免费换新/退货，给您带来不便深表歉意，感谢您的监督。</t>
+          <t>您好，感谢您的反馈。关于“货不对版”问题，我们已记录并将核对仓储记录并补发正确商品，给您带来不便深表歉意，感谢您的监督。</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>非常理解您的心情，质量差确实让人失望。我们已加急处理，会安排质检复核并支持免费换新/退货，希望能再给我们一次弥补的机会～</t>
+          <t>非常理解您的心情，货不对版确实让人失望。我们已加急处理，会核对仓储记录并补发正确商品，希望能再给我们一次弥补的机会～</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>哎呀让您踩坑了！质量差这锅我们背，已安排安排质检复核并支持免费换新/退货，小客服在线等您验收，祝您接下来体验加分～</t>
+          <t>哎呀让您踩坑了！货不对版这锅我们背，已安排核对仓储记录并补发正确商品，小客服在线等您验收，祝您接下来体验加分～</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>bge</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3336,15 +3336,15 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>质量差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.35</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>质量差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -3354,22 +3354,22 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>您好，感谢您的反馈。关于“质量差”问题，我们已记录并将安排质检复核并支持免费换新/退货，给您带来不便深表歉意，感谢您的监督。</t>
+          <t>您好，感谢您的反馈。关于“货不对版”问题，我们已记录并将核对仓储记录并补发正确商品，给您带来不便深表歉意，感谢您的监督。</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>非常理解您的心情，质量差确实让人失望。我们已加急处理，会安排质检复核并支持免费换新/退货，希望能再给我们一次弥补的机会～</t>
+          <t>非常理解您的心情，货不对版确实让人失望。我们已加急处理，会核对仓储记录并补发正确商品，希望能再给我们一次弥补的机会～</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>哎呀让您踩坑了！质量差这锅我们背，已安排安排质检复核并支持免费换新/退货，小客服在线等您验收，祝您接下来体验加分～</t>
+          <t>哎呀让您踩坑了！货不对版这锅我们背，已安排核对仓储记录并补发正确商品，小客服在线等您验收，祝您接下来体验加分～</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>bge</t>
         </is>
       </c>
     </row>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3634,7 +3634,7 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0.67</v>
+        <v>0.706</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3740,7 +3740,7 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3764,7 +3764,7 @@
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0.67</v>
+        <v>0.677</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -3866,15 +3866,15 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>客服态度差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.67</v>
+        <v>0.641</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>客服态度差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -3884,22 +3884,22 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>您好，感谢您的反馈。关于“客服态度差”问题，我们已记录并将对客服进行培训并由主管1小时内回访您，给您带来不便深表歉意，感谢您的监督。</t>
+          <t>您好，感谢您的反馈。关于“货不对版”问题，我们已记录并将核对仓储记录并补发正确商品，给您带来不便深表歉意，感谢您的监督。</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>非常理解您的心情，客服态度差确实让人失望。我们已加急处理，会对客服进行培训并由主管1小时内回访您，希望能再给我们一次弥补的机会～</t>
+          <t>非常理解您的心情，货不对版确实让人失望。我们已加急处理，会核对仓储记录并补发正确商品，希望能再给我们一次弥补的机会～</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>哎呀让您踩坑了！客服态度差这锅我们背，已安排对客服进行培训并由主管1小时内回访您，小客服在线等您验收，祝您接下来体验加分～</t>
+          <t>哎呀让您踩坑了！货不对版这锅我们背，已安排核对仓储记录并补发正确商品，小客服在线等您验收，祝您接下来体验加分～</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>bge</t>
         </is>
       </c>
     </row>
@@ -4005,7 +4005,7 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4164,7 +4164,7 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4217,7 +4217,7 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>0.67</v>
+        <v>0.678</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4323,7 +4323,7 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4376,7 +4376,7 @@
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4429,7 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4555,15 +4555,15 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>客服态度差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.67</v>
+        <v>0.63</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>客服态度差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4573,22 +4573,22 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>您好，感谢您的反馈。关于“客服态度差”问题，我们已记录并将对客服进行培训并由主管1小时内回访您，给您带来不便深表歉意，感谢您的监督。</t>
+          <t>您好，感谢您的反馈。关于“货不对版”问题，我们已记录并将核对仓储记录并补发正确商品，给您带来不便深表歉意，感谢您的监督。</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>非常理解您的心情，客服态度差确实让人失望。我们已加急处理，会对客服进行培训并由主管1小时内回访您，希望能再给我们一次弥补的机会～</t>
+          <t>非常理解您的心情，货不对版确实让人失望。我们已加急处理，会核对仓储记录并补发正确商品，希望能再给我们一次弥补的机会～</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>哎呀让您踩坑了！客服态度差这锅我们背，已安排对客服进行培训并由主管1小时内回访您，小客服在线等您验收，祝您接下来体验加分～</t>
+          <t>哎呀让您踩坑了！货不对版这锅我们背，已安排核对仓储记录并补发正确商品，小客服在线等您验收，祝您接下来体验加分～</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>bge</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>0.67</v>
+        <v>0.675</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4718,7 +4718,7 @@
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>0.79</v>
+        <v>0.791</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4747,7 +4747,7 @@
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4800,7 @@
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4853,7 +4853,7 @@
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -4926,15 +4926,15 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>质量差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>0.67</v>
+        <v>0.649</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>质量差</t>
+          <t>货不对版</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -4944,22 +4944,22 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>您好，感谢您的反馈。关于“质量差”问题，我们已记录并将安排质检复核并支持免费换新/退货，给您带来不便深表歉意，感谢您的监督。</t>
+          <t>您好，感谢您的反馈。关于“货不对版”问题，我们已记录并将核对仓储记录并补发正确商品，给您带来不便深表歉意，感谢您的监督。</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>非常理解您的心情，质量差确实让人失望。我们已加急处理，会安排质检复核并支持免费换新/退货，希望能再给我们一次弥补的机会～</t>
+          <t>非常理解您的心情，货不对版确实让人失望。我们已加急处理，会核对仓储记录并补发正确商品，希望能再给我们一次弥补的机会～</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>哎呀让您踩坑了！质量差这锅我们背，已安排安排质检复核并支持免费换新/退货，小客服在线等您验收，祝您接下来体验加分～</t>
+          <t>哎呀让您踩坑了！货不对版这锅我们背，已安排核对仓储记录并补发正确商品，小客服在线等您验收，祝您接下来体验加分～</t>
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>bge</t>
         </is>
       </c>
     </row>
@@ -5012,7 +5012,7 @@
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5089,7 +5089,7 @@
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>0.35</v>
+        <v>0.573</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5118,7 +5118,7 @@
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5224,7 +5224,7 @@
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5277,7 @@
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5354,7 @@
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>0.35</v>
+        <v>0.556</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5436,7 @@
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5489,7 @@
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5542,7 +5542,7 @@
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5754,7 +5754,7 @@
       </c>
       <c r="K100" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>hybrid-agree</t>
         </is>
       </c>
     </row>
@@ -5856,7 +5856,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"质量差": 30, "客服态度差": 24, "物流慢": 25, "货不对版": 21}</t>
+          <t>{"质量差": 25, "客服态度差": 20, "物流慢": 25, "货不对版": 30}</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>93.0%</t>
+          <t>88.0%</t>
         </is>
       </c>
     </row>
@@ -5892,7 +5892,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>10.83</t>
         </is>
       </c>
     </row>
@@ -5904,7 +5904,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.108</t>
         </is>
       </c>
     </row>

</xml_diff>